<commit_message>
Added component to marble library
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.sahetapy\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230043D4-59DB-4FBE-9BC0-AB9A28EC9CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF6B926-266A-45C5-8B65-E53E055E3D53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
   <si>
     <t>Part Number</t>
   </si>
@@ -79,13 +79,118 @@
   </si>
   <si>
     <t>Library Path</t>
+  </si>
+  <si>
+    <t>SK12D07VG4</t>
+  </si>
+  <si>
+    <t>0.3A @ 30 VDC</t>
+  </si>
+  <si>
+    <t>Slide Switches - Side Knob</t>
+  </si>
+  <si>
+    <t>https://www.snapeda.com/parts/SK12D07VG4/C&amp;K/datasheet/</t>
+  </si>
+  <si>
+    <t>SCH/SK12D07VG4.SchLib</t>
+  </si>
+  <si>
+    <t>PCB/SK12D07VG4.PcbLib</t>
+  </si>
+  <si>
+    <t>1N5819HW-7-F</t>
+  </si>
+  <si>
+    <t>Vf = 450 mV</t>
+  </si>
+  <si>
+    <t>Schottky Diodes &amp; Rectifiers SOD-123</t>
+  </si>
+  <si>
+    <t>SOD3715X145N</t>
+  </si>
+  <si>
+    <t>PCB/SOD3715X145N.PcbLib</t>
+  </si>
+  <si>
+    <t>SCH/1N5819HW-7-F.SchLib</t>
+  </si>
+  <si>
+    <t>https://4donline.ihs.com/images/VipMasterIC/IC/DIOD/DIOD-S-A0011437026/DIOD-S-A0011683586-1.pdf?hkey=CECEF36DEECDED6468708AAF2E19C0C6</t>
+  </si>
+  <si>
+    <t>PJ-002A</t>
+  </si>
+  <si>
+    <t>2.5A @ 24 VDC</t>
+  </si>
+  <si>
+    <t>DC Power Connectors Power Jacks 2x5.5mm</t>
+  </si>
+  <si>
+    <t>CUI_PJ-002A</t>
+  </si>
+  <si>
+    <t>SCH/PJ-002A.SchLib</t>
+  </si>
+  <si>
+    <t>PCB/CUI_PJ-002A.PcbLib</t>
+  </si>
+  <si>
+    <t>https://www.sameskydevices.com/product/resource/pj-002a.pdf</t>
+  </si>
+  <si>
+    <t>Switch Tactile Button 12x12mm</t>
+  </si>
+  <si>
+    <t>FP-MJTP1212A-MFG</t>
+  </si>
+  <si>
+    <t>SCH/button_12mm.SchLib</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/omron-electronics-inc-emc-div/B3F-4055/31799?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=19971370784&amp;gbraid=0AAAAADrbLlgb8g5iB56Pq7GBfmlW8M2um&amp;gclid=CjwKCAiA2svIBhB-EiwARWDPjsxJrtH3aqZi4wzUZvXY0ugmwA-CuPqPru_7AumdmvXcQLZq2TM71hoCQyEQAvD_BwE</t>
+  </si>
+  <si>
+    <t>PCB/button_12mm.PcbLib</t>
+  </si>
+  <si>
+    <t>CMP-47024-000003-1</t>
+  </si>
+  <si>
+    <t>BSS84W-7-F</t>
+  </si>
+  <si>
+    <t>0 V 130mA</t>
+  </si>
+  <si>
+    <t>MOSFET P-Channel 50V 130MA SOT323</t>
+  </si>
+  <si>
+    <t>SOT65P222X110-3N</t>
+  </si>
+  <si>
+    <t>SCH/BSS84W-7-F.SchLib</t>
+  </si>
+  <si>
+    <t>PCB/SOT65P222X110-3N.PcbLib</t>
+  </si>
+  <si>
+    <t>https://www.diodes.com/assets/Datasheets/BSS84W.pdf</t>
+  </si>
+  <si>
+    <t>MJTP1212A</t>
+  </si>
+  <si>
+    <t>0.05A @ 12VDC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -105,6 +210,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -476,18 +587,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" customWidth="1"/>
     <col min="4" max="4" width="84.5703125" customWidth="1"/>
     <col min="5" max="5" width="13.42578125" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" customWidth="1"/>
-    <col min="10" max="10" width="20.85546875" customWidth="1"/>
-    <col min="11" max="11" width="96.42578125" customWidth="1"/>
+    <col min="7" max="7" width="27.42578125" customWidth="1"/>
+    <col min="8" max="8" width="33.5703125" customWidth="1"/>
+    <col min="9" max="9" width="30.140625" customWidth="1"/>
+    <col min="10" max="10" width="43" customWidth="1"/>
+    <col min="11" max="11" width="136.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
@@ -560,9 +673,190 @@
         <v>11</v>
       </c>
     </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-20</v>
+      </c>
+      <c r="F3" s="2">
+        <v>70</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="2">
+        <v>-65</v>
+      </c>
+      <c r="F4" s="2">
+        <v>125</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="2">
+        <v>-25</v>
+      </c>
+      <c r="F5" s="2">
+        <v>85</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="2">
+        <v>-25</v>
+      </c>
+      <c r="F6" s="2">
+        <v>70</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-55</v>
+      </c>
+      <c r="F7" s="2">
+        <v>150</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="K2" r:id="rId1" xr:uid="{62464DCE-AF39-4603-AA20-32EE7D0AF916}"/>
+    <hyperlink ref="K3" r:id="rId2" xr:uid="{3FCFAC1E-539B-45DA-A95A-A3E2C9FBD5DE}"/>
+    <hyperlink ref="K4" r:id="rId3" xr:uid="{68653B32-FEC9-4DDA-9148-9C376AE5E821}"/>
+    <hyperlink ref="K5" r:id="rId4" xr:uid="{61CA21C5-C988-48A1-A8A2-F9FD15B491E5}"/>
+    <hyperlink ref="K6" r:id="rId5" display="https://www.digikey.de/de/products/detail/omron-electronics-inc-emc-div/B3F-4055/31799?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=19971370784&amp;gbraid=0AAAAADrbLlgb8g5iB56Pq7GBfmlW8M2um&amp;gclid=CjwKCAiA2svIBhB-EiwARWDPjsxJrtH3aqZi4wzUZvXY0ugmwA-CuPqPru_7AumdmvXcQLZq2TM71hoCQyEQAvD_BwE" xr:uid="{E4FF004C-5A6C-4B6D-9D01-B58BD91062E9}"/>
+    <hyperlink ref="K7" r:id="rId6" xr:uid="{78F5BECE-FB68-4FD0-9323-150479BC1E56}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added TFT-ST7735 TFT LCD
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.sahetapy\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B146A557-C6A1-4B28-A7C6-5A91FFD510DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96BDD44A-0658-4A2C-B2C8-79C647A48728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="67">
   <si>
     <t>Part Number</t>
   </si>
@@ -205,6 +205,27 @@
   </si>
   <si>
     <t>https://www.snapeda.com/parts/ESP32-DEVKIT-V1/Do+it/view-part/?ref=eda</t>
+  </si>
+  <si>
+    <t>TFT-ST7735</t>
+  </si>
+  <si>
+    <t>1.8 Inch 128x160</t>
+  </si>
+  <si>
+    <t>1.8 inches 128x160 RGB TFT LCD - ST7735 DRIVER</t>
+  </si>
+  <si>
+    <t>ST7735</t>
+  </si>
+  <si>
+    <t>SCH/TFT-ST7735.SchLib</t>
+  </si>
+  <si>
+    <t>PCB/TFT-ST7735.PcbLib</t>
+  </si>
+  <si>
+    <t>https://grabcad.com/library/1-8-inches-128x160-rgb-tft-lcd-st7735-driver-1</t>
   </si>
 </sst>
 </file>
@@ -611,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -907,6 +928,41 @@
         <v>59</v>
       </c>
     </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-30</v>
+      </c>
+      <c r="F9" s="2">
+        <v>80</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
@@ -917,6 +973,7 @@
     <hyperlink ref="K6" r:id="rId5" display="https://www.digikey.de/de/products/detail/omron-electronics-inc-emc-div/B3F-4055/31799?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=19971370784&amp;gbraid=0AAAAADrbLlgb8g5iB56Pq7GBfmlW8M2um&amp;gclid=CjwKCAiA2svIBhB-EiwARWDPjsxJrtH3aqZi4wzUZvXY0ugmwA-CuPqPru_7AumdmvXcQLZq2TM71hoCQyEQAvD_BwE" xr:uid="{E4FF004C-5A6C-4B6D-9D01-B58BD91062E9}"/>
     <hyperlink ref="K7" r:id="rId6" xr:uid="{78F5BECE-FB68-4FD0-9323-150479BC1E56}"/>
     <hyperlink ref="K8" r:id="rId7" xr:uid="{229173BB-844E-4007-BA9D-092EC23AECD2}"/>
+    <hyperlink ref="K9" r:id="rId8" xr:uid="{9E9D47BF-0437-4F4E-877C-47565310CD1B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added ESP32-WROOM-32 to Library
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.sahetapy\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96BDD44A-0658-4A2C-B2C8-79C647A48728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A3F639-23F1-4136-ABAC-D72680F02114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1608" yWindow="17172" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
   <si>
     <t>Part Number</t>
   </si>
@@ -226,6 +226,24 @@
   </si>
   <si>
     <t>https://grabcad.com/library/1-8-inches-128x160-rgb-tft-lcd-st7735-driver-1</t>
+  </si>
+  <si>
+    <t>ESP32-WROOM-32</t>
+  </si>
+  <si>
+    <t>Bluetooth, WiFi 802.11b/g/n, Bluetooth v4.2 +EDR, Class 1, 2 and 3 Transceiver Module U.FL Surface Mount</t>
+  </si>
+  <si>
+    <t>SCH/ESP32-WROOM-32.SchLib</t>
+  </si>
+  <si>
+    <t>MODULE_ESP32-WROOM-32</t>
+  </si>
+  <si>
+    <t>PCB/MODULE_ESP32-WROOM-32.PcbLib</t>
+  </si>
+  <si>
+    <t>https://documentation.espressif.com/esp32-wroom-32_datasheet_en.pdf</t>
   </si>
 </sst>
 </file>
@@ -632,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -963,6 +981,41 @@
         <v>66</v>
       </c>
     </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-40</v>
+      </c>
+      <c r="F10" s="2">
+        <v>85</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
@@ -974,6 +1027,7 @@
     <hyperlink ref="K7" r:id="rId6" xr:uid="{78F5BECE-FB68-4FD0-9323-150479BC1E56}"/>
     <hyperlink ref="K8" r:id="rId7" xr:uid="{229173BB-844E-4007-BA9D-092EC23AECD2}"/>
     <hyperlink ref="K9" r:id="rId8" xr:uid="{9E9D47BF-0437-4F4E-877C-47565310CD1B}"/>
+    <hyperlink ref="K10" r:id="rId9" xr:uid="{1FE31FC4-2FC8-4A7C-8E01-2B38FA19CB9B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added EC11 Rotary Encoder with switch to MarbleLib
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.sahetapy\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A3F639-23F1-4136-ABAC-D72680F02114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29EB599E-25E3-453D-85BE-A47896BCBD93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1608" yWindow="17172" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="80">
   <si>
     <t>Part Number</t>
   </si>
@@ -244,6 +244,27 @@
   </si>
   <si>
     <t>https://documentation.espressif.com/esp32-wroom-32_datasheet_en.pdf</t>
+  </si>
+  <si>
+    <t>EC11E15244G1</t>
+  </si>
+  <si>
+    <t>10mA 5V DC</t>
+  </si>
+  <si>
+    <t>EC11 Rotary Encoder with Switch</t>
+  </si>
+  <si>
+    <t>SCH/EC11E15244G1.SchLib</t>
+  </si>
+  <si>
+    <t>EC11E15244G1_AAL</t>
+  </si>
+  <si>
+    <t>PCB/EC11E15244G1.PcbLib</t>
+  </si>
+  <si>
+    <t>https://tech.alpsalpine.com/e/products/detail/EC11E15244G1/</t>
   </si>
 </sst>
 </file>
@@ -650,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -1016,6 +1037,41 @@
         <v>72</v>
       </c>
     </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="2">
+        <v>-40</v>
+      </c>
+      <c r="F11" s="2">
+        <v>85</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
@@ -1028,6 +1084,7 @@
     <hyperlink ref="K8" r:id="rId7" xr:uid="{229173BB-844E-4007-BA9D-092EC23AECD2}"/>
     <hyperlink ref="K9" r:id="rId8" xr:uid="{9E9D47BF-0437-4F4E-877C-47565310CD1B}"/>
     <hyperlink ref="K10" r:id="rId9" xr:uid="{1FE31FC4-2FC8-4A7C-8E01-2B38FA19CB9B}"/>
+    <hyperlink ref="K11" r:id="rId10" xr:uid="{EF1685DD-C66B-4F3A-84B9-17CB22640930}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added C and R into MarbleLib
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.sahetapy\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DF8577-26DB-4FBB-AB83-A253EEB98666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F2C4CD7-3725-435F-9649-A9CE5D891F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21705" yWindow="-12390" windowWidth="21810" windowHeight="18945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2775" yWindow="3180" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="104">
   <si>
     <t>Part Number</t>
   </si>
@@ -309,19 +309,34 @@
     <t>Capacitor 0805</t>
   </si>
   <si>
-    <t>ECHU1H101JX5</t>
-  </si>
-  <si>
-    <t>SCH/ECHU1H101JX5.SchLib</t>
-  </si>
-  <si>
-    <t>CAP_ECHU1H101JX5</t>
-  </si>
-  <si>
-    <t>PCB/CAP_ECHU1H101JX5.PcbLib</t>
-  </si>
-  <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>CAP0805</t>
+  </si>
+  <si>
+    <t>PCB/Capacitor0805.PcbLib</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>SCH/C.SchLib</t>
+  </si>
+  <si>
+    <t>Resistor 1206</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>SCH/R.SchLib</t>
+  </si>
+  <si>
+    <t>RES1206</t>
+  </si>
+  <si>
+    <t>PCB/Resistor1206.PcbLib</t>
   </si>
 </sst>
 </file>
@@ -728,7 +743,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -1213,25 +1228,60 @@
         <v>93</v>
       </c>
       <c r="E14" s="2">
-        <v>-40</v>
+        <v>-55</v>
       </c>
       <c r="F14" s="2">
         <v>125</v>
       </c>
       <c r="G14" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="K14" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="K14" s="5" t="s">
-        <v>98</v>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1206</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="2">
+        <v>-55</v>
+      </c>
+      <c r="F15" s="2">
+        <v>125</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1250,6 +1300,7 @@
     <hyperlink ref="K12" r:id="rId11" xr:uid="{EEB8497E-ED23-4CC8-BD1C-5A3542C6E0B3}"/>
     <hyperlink ref="K13" r:id="rId12" xr:uid="{BBABDB8F-29DB-4F6B-8DC7-5674625D2A1D}"/>
     <hyperlink ref="K14" r:id="rId13" display="https://www.digikey.de/en/products/detail/phoenix-contact/1984659/950852" xr:uid="{4EFC7E68-0237-41AA-A776-4A57A244EA86}"/>
+    <hyperlink ref="K15" r:id="rId14" display="https://www.digikey.de/en/products/detail/phoenix-contact/1984659/950852" xr:uid="{61CEF08A-6466-4F3A-A214-94AA9A82AD1E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added DW02 & 8205A to MarbleLib
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.sahetapy\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F2C4CD7-3725-435F-9649-A9CE5D891F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9701D0-C154-4D42-A0BA-5A7B3740FCC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2775" yWindow="3180" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="117">
   <si>
     <t>Part Number</t>
   </si>
@@ -337,6 +337,45 @@
   </si>
   <si>
     <t>PCB/Resistor1206.PcbLib</t>
+  </si>
+  <si>
+    <t>FS8205A</t>
+  </si>
+  <si>
+    <t>Dual N-Channel Enhancement Mode Power MOSFET</t>
+  </si>
+  <si>
+    <t>https://www.ic-fortune.com/upload/Download/FS8205A-DS-12_EN.pdf</t>
+  </si>
+  <si>
+    <t>SCH/FS8205A.SchLib</t>
+  </si>
+  <si>
+    <t>SOP65P640X120-8N</t>
+  </si>
+  <si>
+    <t>PCB/SOP65P640X120-8N.PcbLib</t>
+  </si>
+  <si>
+    <t>https://www.snapeda.com/parts/DW01A/Fortune%20Semiconductor/datasheet/</t>
+  </si>
+  <si>
+    <t>DW01A</t>
+  </si>
+  <si>
+    <t>SOT-23-6</t>
+  </si>
+  <si>
+    <t>One Cell Lithium-ion/Polymer Battery Protection IC</t>
+  </si>
+  <si>
+    <t>SCH/DW01A.SchLib</t>
+  </si>
+  <si>
+    <t>SOT95P280X145-6N</t>
+  </si>
+  <si>
+    <t>PCB/SOT95P280X145-6N.PcbLib</t>
   </si>
 </sst>
 </file>
@@ -743,7 +782,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -1284,6 +1323,76 @@
         <v>94</v>
       </c>
     </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-55</v>
+      </c>
+      <c r="F16" s="2">
+        <v>150</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" s="2">
+        <v>-40</v>
+      </c>
+      <c r="F17" s="2">
+        <v>85</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
@@ -1301,6 +1410,8 @@
     <hyperlink ref="K13" r:id="rId12" xr:uid="{BBABDB8F-29DB-4F6B-8DC7-5674625D2A1D}"/>
     <hyperlink ref="K14" r:id="rId13" display="https://www.digikey.de/en/products/detail/phoenix-contact/1984659/950852" xr:uid="{4EFC7E68-0237-41AA-A776-4A57A244EA86}"/>
     <hyperlink ref="K15" r:id="rId14" display="https://www.digikey.de/en/products/detail/phoenix-contact/1984659/950852" xr:uid="{61CEF08A-6466-4F3A-A214-94AA9A82AD1E}"/>
+    <hyperlink ref="K16" r:id="rId15" xr:uid="{B77A82F4-3998-4DD2-94A3-B3BFD0326F64}"/>
+    <hyperlink ref="K17" r:id="rId16" xr:uid="{7545D52A-58FE-49A2-8DE5-2E1490FE2768}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added Buck, screen 3.5 to library; -made V2.00 Altium Project
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\r.sahetapy\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\OneDrive\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9701D0-C154-4D42-A0BA-5A7B3740FCC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7AC3D22-D9C9-4A9B-B827-98110FFF669D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="131">
   <si>
     <t>Part Number</t>
   </si>
@@ -376,6 +376,48 @@
   </si>
   <si>
     <t>PCB/SOT95P280X145-6N.PcbLib</t>
+  </si>
+  <si>
+    <t>MP1484EN-LF</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.925V 1 Output 3A</t>
+  </si>
+  <si>
+    <t>Buck Switching Regulator IC Positive Adjustable 0.925V 1 Output 3A 8-SOIC (0.154", 3.90mm Width)</t>
+  </si>
+  <si>
+    <t>SCH/MP1484EN-LF.SchLib</t>
+  </si>
+  <si>
+    <t>SOIC127P600X170-9N</t>
+  </si>
+  <si>
+    <t>PCB/SOIC127P600X170-9N.PcbLib</t>
+  </si>
+  <si>
+    <t>https://www.digikey.at/de/products/detail/monolithic-power-systems-inc/MP1484EN-LF-Z/5291682?srsltid=AfmBOorvZqZweepwF19jqwdCHLwo1ck00ZSGZEtpVPLNX4bN2FRk_ecr</t>
+  </si>
+  <si>
+    <t>TFT-ILI9488</t>
+  </si>
+  <si>
+    <t>3.5-inch TFT LCD (320 × 480)</t>
+  </si>
+  <si>
+    <t>3.5-inch TFT LCD (320 × 480) with ILI9488 driver + XPT2046 resistive touch</t>
+  </si>
+  <si>
+    <t>https://grabcad.com/library/3-5-color-spi-display-based-on-ili9488-chip-1</t>
+  </si>
+  <si>
+    <t>SCH/6130XX11121_61301411121.SchLib</t>
+  </si>
+  <si>
+    <t>PCB/61301411121.PcbLib</t>
+  </si>
+  <si>
+    <t>TFT_3.5_INCH</t>
   </si>
 </sst>
 </file>
@@ -502,9 +544,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Link" xfId="2" builtinId="8"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Zelle überprüfen" xfId="1" builtinId="23"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -782,17 +824,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
     <col min="2" max="2" width="19.85546875" customWidth="1"/>
-    <col min="3" max="3" width="23.7109375" customWidth="1"/>
-    <col min="4" max="4" width="84.5703125" customWidth="1"/>
+    <col min="3" max="3" width="28.140625" customWidth="1"/>
+    <col min="4" max="4" width="90.7109375" customWidth="1"/>
     <col min="5" max="5" width="13.42578125" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" customWidth="1"/>
     <col min="7" max="7" width="27.42578125" customWidth="1"/>
-    <col min="8" max="8" width="33.5703125" customWidth="1"/>
+    <col min="8" max="8" width="45" customWidth="1"/>
     <col min="9" max="9" width="30.140625" customWidth="1"/>
     <col min="10" max="10" width="43" customWidth="1"/>
     <col min="11" max="11" width="136.7109375" customWidth="1"/>
@@ -1391,6 +1433,76 @@
       </c>
       <c r="K17" s="5" t="s">
         <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E18" s="2">
+        <v>-20</v>
+      </c>
+      <c r="F18" s="2">
+        <v>85</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E19" s="2">
+        <v>-30</v>
+      </c>
+      <c r="F19" s="2">
+        <v>85</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I19" s="2">
+        <v>61301411121</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -1412,6 +1524,8 @@
     <hyperlink ref="K15" r:id="rId14" display="https://www.digikey.de/en/products/detail/phoenix-contact/1984659/950852" xr:uid="{61CEF08A-6466-4F3A-A214-94AA9A82AD1E}"/>
     <hyperlink ref="K16" r:id="rId15" xr:uid="{B77A82F4-3998-4DD2-94A3-B3BFD0326F64}"/>
     <hyperlink ref="K17" r:id="rId16" xr:uid="{7545D52A-58FE-49A2-8DE5-2E1490FE2768}"/>
+    <hyperlink ref="K18" r:id="rId17" xr:uid="{1999A819-4DF6-4646-B0EA-9FF9A230FFB5}"/>
+    <hyperlink ref="K19" r:id="rId18" xr:uid="{94A68611-6BDD-45FD-B434-DBCCF4F72442}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added CH340C USB to UART
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\OneDrive\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7AC3D22-D9C9-4A9B-B827-98110FFF669D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F1234B-A6D0-4AD4-83A9-128BAC446898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21660" yWindow="6450" windowWidth="21765" windowHeight="18945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="137">
   <si>
     <t>Part Number</t>
   </si>
@@ -418,6 +418,24 @@
   </si>
   <si>
     <t>TFT_3.5_INCH</t>
+  </si>
+  <si>
+    <t>CH340C</t>
+  </si>
+  <si>
+    <t>USB to serial chip</t>
+  </si>
+  <si>
+    <t>SCH/CH340C.SchLib</t>
+  </si>
+  <si>
+    <t>SOIC127P600X180-16N</t>
+  </si>
+  <si>
+    <t>PCB/SOIC127P600X180-16N.PcbLib</t>
+  </si>
+  <si>
+    <t>https://www.snapeda.com/parts/CH340C/WCH/datasheet/</t>
   </si>
 </sst>
 </file>
@@ -544,9 +562,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Link" xfId="2" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Zelle überprüfen" xfId="1" builtinId="23"/>
+    <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -824,8 +842,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
     <col min="2" max="2" width="19.85546875" customWidth="1"/>
@@ -1503,6 +1521,41 @@
       </c>
       <c r="K19" s="5" t="s">
         <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E20" s="2">
+        <v>-30</v>
+      </c>
+      <c r="F20" s="2">
+        <v>85</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="K20" s="5" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1526,6 +1579,7 @@
     <hyperlink ref="K17" r:id="rId16" xr:uid="{7545D52A-58FE-49A2-8DE5-2E1490FE2768}"/>
     <hyperlink ref="K18" r:id="rId17" xr:uid="{1999A819-4DF6-4646-B0EA-9FF9A230FFB5}"/>
     <hyperlink ref="K19" r:id="rId18" xr:uid="{94A68611-6BDD-45FD-B434-DBCCF4F72442}"/>
+    <hyperlink ref="K20" r:id="rId19" xr:uid="{ACAB057F-4468-4B22-8C93-E8C22D24B65F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added 2pins 2.54 battery connector
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F1234B-A6D0-4AD4-83A9-128BAC446898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E05888A-862C-439D-8D87-8B4ADA3B1A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21660" yWindow="6450" windowWidth="21765" windowHeight="18945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="143">
   <si>
     <t>Part Number</t>
   </si>
@@ -436,6 +436,24 @@
   </si>
   <si>
     <t>https://www.snapeda.com/parts/CH340C/WCH/datasheet/</t>
+  </si>
+  <si>
+    <t>2POS 2.54MM</t>
+  </si>
+  <si>
+    <t>Connector Header Through Hole 2 position 0.100" (2.54mm)</t>
+  </si>
+  <si>
+    <t>SCH/22232021.SchLib</t>
+  </si>
+  <si>
+    <t>CONN_A-6373-02A_MOL</t>
+  </si>
+  <si>
+    <t>PCB/CONN_A-6373-02A_MOL.PcbLib</t>
+  </si>
+  <si>
+    <t>https://www.molex.com/en-us/products/part-detail/0022232021</t>
   </si>
 </sst>
 </file>
@@ -842,7 +860,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.140625" customWidth="1"/>
@@ -1556,6 +1574,41 @@
       </c>
       <c r="K20" s="5" t="s">
         <v>136</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>22232021</v>
+      </c>
+      <c r="B21" s="2">
+        <v>22232021</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="2">
+        <v>-30</v>
+      </c>
+      <c r="F21" s="2">
+        <v>85</v>
+      </c>
+      <c r="G21" s="2">
+        <v>22232021</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="K21" s="5" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1580,6 +1633,7 @@
     <hyperlink ref="K18" r:id="rId17" xr:uid="{1999A819-4DF6-4646-B0EA-9FF9A230FFB5}"/>
     <hyperlink ref="K19" r:id="rId18" xr:uid="{94A68611-6BDD-45FD-B434-DBCCF4F72442}"/>
     <hyperlink ref="K20" r:id="rId19" xr:uid="{ACAB057F-4468-4B22-8C93-E8C22D24B65F}"/>
+    <hyperlink ref="K21" r:id="rId20" xr:uid="{F4194E98-BFEF-4B12-A2C1-854A13CE3C9C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Added USB Type C 6p & 16p into library ; continued schematic for master V2.00
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E05888A-862C-439D-8D87-8B4ADA3B1A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091F2723-497F-45EA-99ED-531C847873CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="159">
   <si>
     <t>Part Number</t>
   </si>
@@ -454,6 +454,54 @@
   </si>
   <si>
     <t>https://www.molex.com/en-us/products/part-detail/0022232021</t>
+  </si>
+  <si>
+    <t>USB4125-GF-A-0190</t>
+  </si>
+  <si>
+    <t>6 Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	CONN RCPT TYPE C 6P SMD RA</t>
+  </si>
+  <si>
+    <t>USB-C 2.0</t>
+  </si>
+  <si>
+    <t>SCH/USB4125-GF-A-0190_REVA2.SchLib</t>
+  </si>
+  <si>
+    <t>GCT_USB4125-GF-A-0190_REVA2</t>
+  </si>
+  <si>
+    <t>PCB/GCT_USB4125-GF-A-0190_REVA2.PcbLib</t>
+  </si>
+  <si>
+    <t>https://gct.co/files/specs/usb4125-spec.pdf</t>
+  </si>
+  <si>
+    <t>USB4105-GF-A-060</t>
+  </si>
+  <si>
+    <t>16 Pin</t>
+  </si>
+  <si>
+    <t>CONN RCP USB2.0 TYP C 16P SMD RA</t>
+  </si>
+  <si>
+    <t>USB Type C 16P</t>
+  </si>
+  <si>
+    <t>SCH/USB4105-GF-A-060.SchLib</t>
+  </si>
+  <si>
+    <t>GCT_USB4105-GF-A-060</t>
+  </si>
+  <si>
+    <t>PCB/GCT_USB4105-GF-A-060.PcbLib</t>
+  </si>
+  <si>
+    <t>https://gct.co/files/specs/usb4105-spec.pdf</t>
   </si>
 </sst>
 </file>
@@ -860,10 +908,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.140625" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
     <col min="2" max="2" width="19.85546875" customWidth="1"/>
     <col min="3" max="3" width="28.140625" customWidth="1"/>
     <col min="4" max="4" width="90.7109375" customWidth="1"/>
@@ -1609,6 +1657,76 @@
       </c>
       <c r="K21" s="5" t="s">
         <v>142</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E22" s="2">
+        <v>-30</v>
+      </c>
+      <c r="F22" s="2">
+        <v>85</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E23" s="2">
+        <v>-40</v>
+      </c>
+      <c r="F23" s="2">
+        <v>85</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -1634,6 +1752,8 @@
     <hyperlink ref="K19" r:id="rId18" xr:uid="{94A68611-6BDD-45FD-B434-DBCCF4F72442}"/>
     <hyperlink ref="K20" r:id="rId19" xr:uid="{ACAB057F-4468-4B22-8C93-E8C22D24B65F}"/>
     <hyperlink ref="K21" r:id="rId20" xr:uid="{F4194E98-BFEF-4B12-A2C1-854A13CE3C9C}"/>
+    <hyperlink ref="K22" r:id="rId21" xr:uid="{BE4EDFA5-F1AC-4169-B5FB-956CDB9ED25F}"/>
+    <hyperlink ref="K23" r:id="rId22" xr:uid="{6AEAE48E-4C59-41F2-BB06-858E00F21DE2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Addded inductor to Lib
</commit_message>
<xml_diff>
--- a/pcb/Library/MarbleLib.xlsx
+++ b/pcb/Library/MarbleLib.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ruben\Documents\Git\Marble-Station-ESP32\pcb\Library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091F2723-497F-45EA-99ED-531C847873CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FDB582-FA21-4FE4-B122-592E25CBA535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21705" yWindow="6450" windowWidth="21810" windowHeight="18945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21600" yWindow="-3405" windowWidth="21810" windowHeight="15930" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Components" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="165">
   <si>
     <t>Part Number</t>
   </si>
@@ -502,6 +502,24 @@
   </si>
   <si>
     <t>https://gct.co/files/specs/usb4105-spec.pdf</t>
+  </si>
+  <si>
+    <t>SRP1038AA-R36M</t>
+  </si>
+  <si>
+    <t>11 mm x 10 mm</t>
+  </si>
+  <si>
+    <t>SMD Inductor 11x10mm</t>
+  </si>
+  <si>
+    <t>SCH/SRP1038AA-R36M.SchLib</t>
+  </si>
+  <si>
+    <t>INDPM110100X400N</t>
+  </si>
+  <si>
+    <t>PCB/INDPM110100X400N.PcbLib</t>
   </si>
 </sst>
 </file>
@@ -908,7 +926,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
@@ -1726,6 +1744,41 @@
         <v>157</v>
       </c>
       <c r="K23" s="5" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E24" s="2">
+        <v>-55</v>
+      </c>
+      <c r="F24" s="2">
+        <v>155</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="K24" s="5" t="s">
         <v>158</v>
       </c>
     </row>
@@ -1754,6 +1807,7 @@
     <hyperlink ref="K21" r:id="rId20" xr:uid="{F4194E98-BFEF-4B12-A2C1-854A13CE3C9C}"/>
     <hyperlink ref="K22" r:id="rId21" xr:uid="{BE4EDFA5-F1AC-4169-B5FB-956CDB9ED25F}"/>
     <hyperlink ref="K23" r:id="rId22" xr:uid="{6AEAE48E-4C59-41F2-BB06-858E00F21DE2}"/>
+    <hyperlink ref="K24" r:id="rId23" xr:uid="{6FD8282A-76A1-4640-B675-63202C847A00}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>